<commit_message>
Add the SkillNavora Handbooks hub (/handbooks/), Tableau track and the expanded Excel lesson; refresh the Data Science & AI handbook (116 lessons, 9 tracks)
- /handbooks/: Data Science & AI, GenAI Launchpad (400-page PDF), DSA and the interactive PM Master Handbook, with every PDF
- /data-science/: 6 new Tableau lessons with PDFs, Excel lesson 7 OFFSET and consolidation, complete PDF in four parts by track
- PM handbook complete PDF also in two parts; menu link Upskill for free -> SkillNavora Handbooks
- Resources: links to the combined handbook artifact and the handbooks hub

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017PtK5YiriwfHtuW98ocpRw
</commit_message>
<xml_diff>
--- a/data-science/files/excel/excel-07.xlsx
+++ b/data-science/files/excel/excel-07.xlsx
@@ -16,7 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. XLOOKUP examples (lookup tab" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. INDEX returns a value at a p" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Two-way lookup =INDEX($B$2$E" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. CHOOSE examples" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Two-way lookup of a share pr" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Consolidation tasks state fr" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. CHOOSE examples" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -499,6 +501,527 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Asha Foods</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Kiran Motors</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Meru Steel</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>INDEX + MATCH</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>OFFSET + MATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B2" t="n">
+        <v>412</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1180</v>
+      </c>
+      <c r="D2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Kiran Motors</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>46112</v>
+      </c>
+      <c r="H2">
+        <f>INDEX($B$2:$D$6,MATCH(G2,$A$2:$A$6,0),MATCH(F2,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>OFFSET($A$1,MATCH(G2,$A$2:$A$6,0),MATCH(F2,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B3" t="n">
+        <v>398</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1215</v>
+      </c>
+      <c r="D3" t="n">
+        <v>101</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Meru Steel</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>46173</v>
+      </c>
+      <c r="H3">
+        <f>INDEX($B$2:$D$6,MATCH(G3,$A$2:$A$6,0),MATCH(F3,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>OFFSET($A$1,MATCH(G3,$A$2:$A$6,0),MATCH(F3,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B4" t="n">
+        <v>425</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1262</v>
+      </c>
+      <c r="D4" t="n">
+        <v>99</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Asha Foods</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>46081</v>
+      </c>
+      <c r="H4">
+        <f>INDEX($B$2:$D$6,MATCH(G4,$A$2:$A$6,0),MATCH(F4,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>OFFSET($A$1,MATCH(G4,$A$2:$A$6,0),MATCH(F4,$B$1:$D$1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B5" t="n">
+        <v>440</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1240</v>
+      </c>
+      <c r="D5" t="n">
+        <v>108</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Last 3 months avg (Asha)</t>
+        </is>
+      </c>
+      <c r="I5">
+        <f>AVERAGE(OFFSET($B$1,COUNT($B$2:$B$6)-2,0,3,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B6" t="n">
+        <v>436</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1298</v>
+      </c>
+      <c r="D6" t="n">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>City Code</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Population 2011 (mn)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>State of this city</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="H2">
+        <f>_xlfn.IFNA(INDEX($C$2:$C$7,MATCH(G2,$B$2:$B$7,0)),"Not found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Population of city code</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>C31</t>
+        </is>
+      </c>
+      <c r="H3">
+        <f>_xlfn.IFNA(INDEX($D$2:$D$7,MATCH(G3,$A$2:$A$7,0)),"Not found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ahmedabad</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gujarat</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Population of city code</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H4">
+        <f>_xlfn.IFNA(INDEX($D$2:$D$7,MATCH(G4,$A$2:$A$7,0)),"Not found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Surat</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gujarat</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>City code of this city</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Allahabad</t>
+        </is>
+      </c>
+      <c r="H5">
+        <f>_xlfn.IFNA(INDEX($A$2:$A$7,MATCH(G5,$B$2:$B$7,0)),"Not found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Allahabad</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Grade (approx. match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <f>VLOOKUP(F8,$F$12:$G$15,2,TRUE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="F9" t="n">
+        <v>58</v>
+      </c>
+      <c r="G9">
+        <f>VLOOKUP(F9,$F$12:$G$15,2,TRUE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="F10" t="n">
+        <v>91</v>
+      </c>
+      <c r="G10">
+        <f>VLOOKUP(F10,$F$12:$G$15,2,TRUE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Min marks</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="F13" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" t="n">
+        <v>60</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="F15" t="n">
+        <v>80</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>